<commit_message>
Update mesh6 reference spreadsheet
</commit_message>
<xml_diff>
--- a/docs/mesh6.xlsx
+++ b/docs/mesh6.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ADATA\LITHIUM\GITHUB\ogs-lithium-model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ADATA\LITHIUM\GITHUB\ogs-lithium-model\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87447779-93F4-4E75-A184-45F46873B721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E451C7A0-D751-41DA-9C5D-CBF254338CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="74">
   <si>
     <t>x</t>
   </si>
@@ -262,66 +262,6 @@
   </si>
   <si>
     <t>Bottom</t>
-  </si>
-  <si>
-    <t>3 101 Layer5_bottom</t>
-  </si>
-  <si>
-    <t>3 102 Layer4_caprock2</t>
-  </si>
-  <si>
-    <t>3 103 Layer3_Reservoir</t>
-  </si>
-  <si>
-    <t>3 104 Layer2_caprock1</t>
-  </si>
-  <si>
-    <t>3 105 Layer1_Top</t>
-  </si>
-  <si>
-    <t>3 201 Well1</t>
-  </si>
-  <si>
-    <t>3 202 Well1_upper</t>
-  </si>
-  <si>
-    <t>3 203 Well1_middle</t>
-  </si>
-  <si>
-    <t>3 204 Well1_bottom</t>
-  </si>
-  <si>
-    <t>3 205 Well2</t>
-  </si>
-  <si>
-    <t>3 206 Well2_upper</t>
-  </si>
-  <si>
-    <t>3 207 Well2_middle</t>
-  </si>
-  <si>
-    <t>3 208 Well2_bottom</t>
-  </si>
-  <si>
-    <t>Length: meters</t>
-  </si>
-  <si>
-    <t>Time: seconds</t>
-  </si>
-  <si>
-    <t>Pressure: Pascal</t>
-  </si>
-  <si>
-    <t>Permeability: m²</t>
-  </si>
-  <si>
-    <t>Viscosity: Pa·s</t>
-  </si>
-  <si>
-    <t>Density: kg/m³</t>
-  </si>
-  <si>
-    <t>Porosity: dimensionless</t>
   </si>
 </sst>
 </file>
@@ -387,7 +327,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -432,12 +372,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="3" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -455,7 +389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -508,58 +442,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -571,11 +463,31 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1021,8 +933,8 @@
     <col min="1" max="8" width="9.7109375" customWidth="1"/>
     <col min="9" max="9" width="14.42578125" customWidth="1"/>
     <col min="10" max="18" width="9.7109375" customWidth="1"/>
-    <col min="19" max="19" width="3.42578125" style="49" customWidth="1"/>
-    <col min="20" max="20" width="10.5703125" style="47" customWidth="1"/>
+    <col min="19" max="19" width="3.42578125" style="32" customWidth="1"/>
+    <col min="20" max="20" width="10.5703125" customWidth="1"/>
     <col min="23" max="23" width="17" customWidth="1"/>
     <col min="24" max="24" width="15.42578125" customWidth="1"/>
     <col min="36" max="36" width="17.140625" customWidth="1"/>
@@ -1047,17 +959,9 @@
         <v>10</v>
       </c>
       <c r="G2" s="8"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="33"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="33"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="R2" s="1"/>
       <c r="U2" s="10" t="s">
         <v>34</v>
       </c>
@@ -1077,18 +981,13 @@
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="34" t="s">
+      <c r="H3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-      <c r="N3" s="33"/>
-      <c r="O3" s="33"/>
-      <c r="P3" s="33"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="33"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="R3" s="1"/>
       <c r="V3" s="13" t="s">
         <v>66</v>
       </c>
@@ -1105,17 +1004,11 @@
       <c r="G4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32"/>
-      <c r="M4" s="33"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="33"/>
-      <c r="Q4" s="32"/>
-      <c r="R4" s="33"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="R4" s="1"/>
       <c r="V4" s="10" t="s">
         <v>43</v>
       </c>
@@ -1135,16 +1028,16 @@
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
-      <c r="H5" s="44" t="s">
+      <c r="H5" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="44" t="s">
+      <c r="I5" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="J5" s="44" t="s">
+      <c r="J5" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="44" t="s">
+      <c r="K5" s="28" t="s">
         <v>9</v>
       </c>
       <c r="AA5" s="10" t="s">
@@ -1175,16 +1068,16 @@
       <c r="G6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="I6" s="45" t="s">
+      <c r="I6" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="J6" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="K6" s="45" t="s">
+      <c r="J6" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" s="29" t="s">
         <v>10</v>
       </c>
       <c r="V6" s="9" t="s">
@@ -1223,10 +1116,10 @@
       <c r="AH6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="AI6" s="30" t="s">
+      <c r="AI6" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="AJ6" s="30"/>
+      <c r="AJ6" s="34"/>
       <c r="AK6" s="9" t="s">
         <v>0</v>
       </c>
@@ -1265,16 +1158,16 @@
       <c r="G7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="46" t="s">
+      <c r="H7" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="46" t="s">
+      <c r="I7" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="J7" s="46" t="s">
+      <c r="J7" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="46" t="s">
+      <c r="K7" s="30" t="s">
         <v>11</v>
       </c>
       <c r="V7" s="5" t="s">
@@ -1293,33 +1186,33 @@
         <v>105</v>
       </c>
       <c r="AA7" s="1">
-        <f>O13</f>
+        <f t="shared" ref="AA7:AC11" si="0">O13</f>
         <v>5</v>
       </c>
       <c r="AB7" s="1">
-        <f>P13</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AC7" s="1">
-        <f>Q13</f>
+        <f t="shared" si="0"/>
         <v>4.25</v>
       </c>
-      <c r="AE7" s="26" t="s">
+      <c r="AE7" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="AF7" s="26" t="s">
+      <c r="AF7" s="35" t="s">
         <v>25</v>
       </c>
       <c r="AG7" s="1">
         <v>3</v>
       </c>
-      <c r="AH7" s="26">
+      <c r="AH7" s="35">
         <v>7</v>
       </c>
-      <c r="AI7" s="29">
+      <c r="AI7" s="33">
         <v>201</v>
       </c>
-      <c r="AJ7" s="29">
+      <c r="AJ7" s="33">
         <v>202</v>
       </c>
       <c r="AK7" s="1">
@@ -1349,7 +1242,7 @@
       <c r="AS7" s="17"/>
     </row>
     <row r="8" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="38" t="s">
         <v>17</v>
       </c>
       <c r="B8" s="4"/>
@@ -1357,16 +1250,16 @@
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
-      <c r="H8" s="45" t="s">
+      <c r="H8" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="45" t="s">
+      <c r="I8" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="45" t="s">
+      <c r="J8" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="45" t="s">
+      <c r="K8" s="29" t="s">
         <v>12</v>
       </c>
       <c r="V8" s="5" t="s">
@@ -1385,25 +1278,25 @@
         <v>104</v>
       </c>
       <c r="AA8" s="1">
-        <f>O14</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AB8" s="1">
-        <f>P14</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AC8" s="1">
-        <f>Q14</f>
+        <f t="shared" si="0"/>
         <v>3.25</v>
       </c>
-      <c r="AE8" s="26"/>
-      <c r="AF8" s="26"/>
+      <c r="AE8" s="35"/>
+      <c r="AF8" s="35"/>
       <c r="AG8" s="1">
         <v>3</v>
       </c>
-      <c r="AH8" s="26"/>
-      <c r="AI8" s="29"/>
-      <c r="AJ8" s="29"/>
+      <c r="AH8" s="35"/>
+      <c r="AI8" s="33"/>
+      <c r="AJ8" s="33"/>
       <c r="AK8" s="1">
         <v>1</v>
       </c>
@@ -1436,22 +1329,22 @@
       </c>
     </row>
     <row r="9" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A9" s="25"/>
+      <c r="A9" s="38"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
-      <c r="H9" s="44" t="s">
+      <c r="H9" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="44" t="s">
+      <c r="I9" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="J9" s="44" t="s">
+      <c r="J9" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="K9" s="44" t="s">
+      <c r="K9" s="28" t="s">
         <v>7</v>
       </c>
       <c r="V9" s="5" t="s">
@@ -1470,25 +1363,25 @@
         <v>103</v>
       </c>
       <c r="AA9" s="1">
-        <f>O15</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AB9" s="1">
-        <f>P15</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AC9" s="1">
-        <f>Q15</f>
+        <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="AE9" s="26"/>
-      <c r="AF9" s="26"/>
+      <c r="AE9" s="35"/>
+      <c r="AF9" s="35"/>
       <c r="AG9" s="1">
         <v>3</v>
       </c>
-      <c r="AH9" s="26"/>
-      <c r="AI9" s="29"/>
-      <c r="AJ9" s="29"/>
+      <c r="AH9" s="35"/>
+      <c r="AI9" s="33"/>
+      <c r="AJ9" s="33"/>
       <c r="AK9" s="1">
         <v>1</v>
       </c>
@@ -1543,29 +1436,29 @@
         <v>102</v>
       </c>
       <c r="AA10" s="1">
-        <f>O16</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AB10" s="1">
-        <f>P16</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AC10" s="1">
-        <f>Q16</f>
+        <f t="shared" si="0"/>
         <v>1.75</v>
       </c>
-      <c r="AE10" s="26"/>
-      <c r="AF10" s="26" t="s">
+      <c r="AE10" s="35"/>
+      <c r="AF10" s="35" t="s">
         <v>26</v>
       </c>
       <c r="AG10" s="1">
         <v>3</v>
       </c>
-      <c r="AH10" s="26">
+      <c r="AH10" s="35">
         <v>10</v>
       </c>
-      <c r="AI10" s="29"/>
-      <c r="AJ10" s="29">
+      <c r="AI10" s="33"/>
+      <c r="AJ10" s="33">
         <v>203</v>
       </c>
       <c r="AK10" s="1">
@@ -1604,22 +1497,22 @@
       <c r="G11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="H11" s="36"/>
-      <c r="I11" s="37" t="s">
-        <v>5</v>
-      </c>
-      <c r="J11" s="37"/>
-      <c r="K11" s="37"/>
-      <c r="L11" s="37" t="s">
+      <c r="H11" s="9"/>
+      <c r="I11" s="39" t="s">
+        <v>5</v>
+      </c>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="M11" s="37"/>
-      <c r="N11" s="37"/>
-      <c r="O11" s="35" t="s">
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="P11" s="35"/>
-      <c r="Q11" s="35"/>
+      <c r="P11" s="34"/>
+      <c r="Q11" s="34"/>
       <c r="V11" s="5" t="s">
         <v>27</v>
       </c>
@@ -1636,25 +1529,25 @@
         <v>101</v>
       </c>
       <c r="AA11" s="1">
-        <f>O17</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AB11" s="1">
-        <f>P17</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="AC11" s="1">
-        <f>Q17</f>
+        <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
-      <c r="AE11" s="26"/>
-      <c r="AF11" s="26"/>
+      <c r="AE11" s="35"/>
+      <c r="AF11" s="35"/>
       <c r="AG11" s="1">
         <v>3</v>
       </c>
-      <c r="AH11" s="26"/>
-      <c r="AI11" s="29"/>
-      <c r="AJ11" s="29"/>
+      <c r="AH11" s="35"/>
+      <c r="AI11" s="33"/>
+      <c r="AJ11" s="33"/>
       <c r="AK11" s="1">
         <v>1</v>
       </c>
@@ -1691,42 +1584,42 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="8"/>
-      <c r="H12" s="31"/>
-      <c r="I12" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="J12" s="36" t="s">
-        <v>1</v>
-      </c>
-      <c r="K12" s="38" t="s">
-        <v>2</v>
-      </c>
-      <c r="L12" s="39" t="s">
+      <c r="H12" s="10"/>
+      <c r="I12" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="K12" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="L12" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="M12" s="40" t="s">
+      <c r="M12" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="N12" s="38" t="s">
+      <c r="N12" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="O12" s="39" t="s">
+      <c r="O12" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="P12" s="40" t="s">
+      <c r="P12" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="Q12" s="38" t="s">
+      <c r="Q12" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="AE12" s="26"/>
-      <c r="AF12" s="26"/>
+      <c r="AE12" s="35"/>
+      <c r="AF12" s="35"/>
       <c r="AG12" s="1">
         <v>3</v>
       </c>
-      <c r="AH12" s="26"/>
-      <c r="AI12" s="29"/>
-      <c r="AJ12" s="29"/>
+      <c r="AH12" s="35"/>
+      <c r="AI12" s="33"/>
+      <c r="AJ12" s="33"/>
       <c r="AK12" s="1">
         <v>1</v>
       </c>
@@ -1763,55 +1656,55 @@
       <c r="G13" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H13" s="48" t="s">
+      <c r="H13" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="I13" s="33">
-        <v>0</v>
-      </c>
-      <c r="J13" s="33">
-        <v>0</v>
-      </c>
-      <c r="K13" s="41">
-        <v>5</v>
-      </c>
-      <c r="L13" s="42">
-        <f t="shared" ref="L13:L18" si="0">$C$2</f>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0</v>
+      </c>
+      <c r="K13" s="27">
+        <v>5</v>
+      </c>
+      <c r="L13" s="6">
+        <f t="shared" ref="L13:L18" si="1">$C$2</f>
         <v>10</v>
       </c>
-      <c r="M13" s="43">
-        <f t="shared" ref="M13:M18" si="1">$F$2</f>
+      <c r="M13" s="7">
+        <f t="shared" ref="M13:M18" si="2">$F$2</f>
         <v>10</v>
       </c>
-      <c r="N13" s="41">
+      <c r="N13" s="27">
         <f>K13-K14</f>
         <v>1.5</v>
       </c>
-      <c r="O13" s="39">
+      <c r="O13" s="25">
         <f>L13/2</f>
         <v>5</v>
       </c>
-      <c r="P13" s="40">
+      <c r="P13" s="26">
         <f>M13/2</f>
         <v>5</v>
       </c>
-      <c r="Q13" s="38">
+      <c r="Q13" s="24">
         <f>(N13/2)+K14</f>
         <v>4.25</v>
       </c>
       <c r="AA13" s="17"/>
-      <c r="AE13" s="26"/>
-      <c r="AF13" s="26" t="s">
+      <c r="AE13" s="35"/>
+      <c r="AF13" s="35" t="s">
         <v>27</v>
       </c>
       <c r="AG13" s="1">
         <v>3</v>
       </c>
-      <c r="AH13" s="26">
+      <c r="AH13" s="35">
         <v>13</v>
       </c>
-      <c r="AI13" s="29"/>
-      <c r="AJ13" s="29">
+      <c r="AI13" s="33"/>
+      <c r="AJ13" s="33">
         <v>204</v>
       </c>
       <c r="AK13" s="1">
@@ -1841,54 +1734,54 @@
       <c r="AS13" s="16"/>
     </row>
     <row r="14" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="H14" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="I14" s="33">
-        <v>0</v>
-      </c>
-      <c r="J14" s="33">
-        <v>0</v>
-      </c>
-      <c r="K14" s="41">
+      <c r="H14" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="I14" s="1">
+        <v>0</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="27">
         <v>3.5</v>
       </c>
-      <c r="L14" s="42">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="M14" s="43">
+      <c r="L14" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N14" s="41">
+      <c r="M14" s="7">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="N14" s="27">
         <f>K14-K15</f>
         <v>0.5</v>
       </c>
-      <c r="O14" s="39">
-        <f t="shared" ref="O14:O18" si="2">L14/2</f>
-        <v>5</v>
-      </c>
-      <c r="P14" s="40">
-        <f t="shared" ref="P14:P18" si="3">M14/2</f>
-        <v>5</v>
-      </c>
-      <c r="Q14" s="38">
-        <f t="shared" ref="Q14:Q16" si="4">(N14/2)+K15</f>
+      <c r="O14" s="25">
+        <f t="shared" ref="O14:O18" si="3">L14/2</f>
+        <v>5</v>
+      </c>
+      <c r="P14" s="26">
+        <f t="shared" ref="P14:P18" si="4">M14/2</f>
+        <v>5</v>
+      </c>
+      <c r="Q14" s="24">
+        <f t="shared" ref="Q14:Q16" si="5">(N14/2)+K15</f>
         <v>3.25</v>
       </c>
       <c r="V14" s="13" t="s">
         <v>53</v>
       </c>
       <c r="AA14" s="17"/>
-      <c r="AE14" s="26"/>
-      <c r="AF14" s="26"/>
+      <c r="AE14" s="35"/>
+      <c r="AF14" s="35"/>
       <c r="AG14" s="1">
         <v>3</v>
       </c>
-      <c r="AH14" s="26"/>
-      <c r="AI14" s="29"/>
-      <c r="AJ14" s="29"/>
+      <c r="AH14" s="35"/>
+      <c r="AI14" s="33"/>
+      <c r="AJ14" s="33"/>
       <c r="AK14" s="1">
         <v>1</v>
       </c>
@@ -1924,53 +1817,53 @@
       <c r="B15" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H15" s="48" t="s">
+      <c r="H15" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="I15" s="33">
-        <v>0</v>
-      </c>
-      <c r="J15" s="33">
-        <v>0</v>
-      </c>
-      <c r="K15" s="41">
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0</v>
+      </c>
+      <c r="K15" s="27">
         <v>3</v>
       </c>
-      <c r="L15" s="42">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="M15" s="43">
+      <c r="L15" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N15" s="41">
+      <c r="M15" s="7">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="N15" s="27">
         <f>K15-K16</f>
         <v>1</v>
       </c>
-      <c r="O15" s="39">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="P15" s="40">
+      <c r="O15" s="25">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="Q15" s="38">
+      <c r="P15" s="26">
         <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="Q15" s="24">
+        <f t="shared" si="5"/>
         <v>2.5</v>
       </c>
       <c r="V15" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="AE15" s="26"/>
-      <c r="AF15" s="26"/>
+      <c r="AE15" s="35"/>
+      <c r="AF15" s="35"/>
       <c r="AG15" s="1">
         <v>3</v>
       </c>
-      <c r="AH15" s="26"/>
-      <c r="AI15" s="29"/>
-      <c r="AJ15" s="29"/>
+      <c r="AH15" s="35"/>
+      <c r="AI15" s="33"/>
+      <c r="AJ15" s="33"/>
       <c r="AK15" s="1">
         <v>1</v>
       </c>
@@ -2004,40 +1897,40 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-      <c r="H16" s="48" t="s">
+      <c r="H16" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="I16" s="33">
-        <v>0</v>
-      </c>
-      <c r="J16" s="33">
-        <v>0</v>
-      </c>
-      <c r="K16" s="41">
-        <v>2</v>
-      </c>
-      <c r="L16" s="42">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="M16" s="43">
+      <c r="I16" s="1">
+        <v>0</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="27">
+        <v>2</v>
+      </c>
+      <c r="L16" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N16" s="41">
+      <c r="M16" s="7">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="N16" s="27">
         <f>K16-K17</f>
         <v>0.5</v>
       </c>
-      <c r="O16" s="39">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="P16" s="40">
+      <c r="O16" s="25">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="Q16" s="38">
+      <c r="P16" s="26">
         <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="Q16" s="24">
+        <f t="shared" si="5"/>
         <v>1.75</v>
       </c>
       <c r="Z16" s="17"/>
@@ -2046,22 +1939,22 @@
       </c>
       <c r="AB16" s="10"/>
       <c r="AC16" s="10"/>
-      <c r="AE16" s="26" t="s">
+      <c r="AE16" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="AF16" s="26" t="s">
+      <c r="AF16" s="35" t="s">
         <v>25</v>
       </c>
       <c r="AG16" s="1">
         <v>3</v>
       </c>
-      <c r="AH16" s="26">
+      <c r="AH16" s="35">
         <v>8</v>
       </c>
-      <c r="AI16" s="29">
+      <c r="AI16" s="33">
         <v>205</v>
       </c>
-      <c r="AJ16" s="29">
+      <c r="AJ16" s="33">
         <v>206</v>
       </c>
       <c r="AK16" s="1">
@@ -2096,39 +1989,39 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="H17" s="48" t="s">
+      <c r="H17" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="33">
-        <v>0</v>
-      </c>
-      <c r="J17" s="33">
-        <v>0</v>
-      </c>
-      <c r="K17" s="41">
+      <c r="I17" s="1">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="27">
         <v>1.5</v>
       </c>
-      <c r="L17" s="42">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="M17" s="43">
+      <c r="L17" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N17" s="41">
+      <c r="M17" s="7">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="N17" s="27">
         <f>K17-K18</f>
         <v>1.5</v>
       </c>
-      <c r="O17" s="39">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="P17" s="40">
+      <c r="O17" s="25">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="Q17" s="38">
+      <c r="P17" s="26">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="Q17" s="24">
         <f>(N17/2)+K18</f>
         <v>0.75</v>
       </c>
@@ -2156,14 +2049,14 @@
       <c r="AC17" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AE17" s="26"/>
-      <c r="AF17" s="26"/>
+      <c r="AE17" s="35"/>
+      <c r="AF17" s="35"/>
       <c r="AG17" s="1">
         <v>3</v>
       </c>
-      <c r="AH17" s="26"/>
-      <c r="AI17" s="29"/>
-      <c r="AJ17" s="29"/>
+      <c r="AH17" s="35"/>
+      <c r="AI17" s="33"/>
+      <c r="AJ17" s="33"/>
       <c r="AK17" s="1">
         <v>9</v>
       </c>
@@ -2201,46 +2094,46 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="H18" s="48" t="s">
+      <c r="H18" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="I18" s="33">
-        <v>0</v>
-      </c>
-      <c r="J18" s="33">
-        <v>0</v>
-      </c>
-      <c r="K18" s="41">
-        <v>0</v>
-      </c>
-      <c r="L18" s="42">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="M18" s="43">
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>0</v>
+      </c>
+      <c r="K18" s="27">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N18" s="41">
+      <c r="M18" s="7">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="N18" s="27">
         <f>K18</f>
         <v>0</v>
       </c>
-      <c r="O18" s="39">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="P18" s="40">
+      <c r="O18" s="25">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="Q18" s="38">
-        <f t="shared" ref="Q18" si="5">N18/2</f>
-        <v>0</v>
-      </c>
-      <c r="V18" s="27" t="s">
+      <c r="P18" s="26">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="Q18" s="24">
+        <f t="shared" ref="Q18" si="6">N18/2</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="W18" s="28" t="s">
+      <c r="W18" s="37" t="s">
         <v>54</v>
       </c>
       <c r="X18" s="1">
@@ -2249,7 +2142,7 @@
       <c r="Y18" s="1">
         <v>1</v>
       </c>
-      <c r="Z18" s="29">
+      <c r="Z18" s="33">
         <v>301</v>
       </c>
       <c r="AA18" s="1">
@@ -2261,14 +2154,14 @@
       <c r="AC18" s="1">
         <v>4.25</v>
       </c>
-      <c r="AE18" s="26"/>
-      <c r="AF18" s="26"/>
+      <c r="AE18" s="35"/>
+      <c r="AF18" s="35"/>
       <c r="AG18" s="1">
         <v>3</v>
       </c>
-      <c r="AH18" s="26"/>
-      <c r="AI18" s="29"/>
-      <c r="AJ18" s="29"/>
+      <c r="AH18" s="35"/>
+      <c r="AI18" s="33"/>
+      <c r="AJ18" s="33"/>
       <c r="AK18" s="1">
         <v>9</v>
       </c>
@@ -2305,25 +2198,16 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="32"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-      <c r="N19" s="32"/>
-      <c r="O19" s="33"/>
-      <c r="P19" s="32"/>
-      <c r="Q19" s="32"/>
-      <c r="V19" s="27"/>
-      <c r="W19" s="28"/>
+      <c r="O19" s="1"/>
+      <c r="V19" s="36"/>
+      <c r="W19" s="37"/>
       <c r="X19" s="14">
         <v>2</v>
       </c>
       <c r="Y19" s="1">
         <v>13</v>
       </c>
-      <c r="Z19" s="29"/>
+      <c r="Z19" s="33"/>
       <c r="AA19" s="1">
         <v>0</v>
       </c>
@@ -2333,18 +2217,18 @@
       <c r="AC19" s="1">
         <v>3.25</v>
       </c>
-      <c r="AE19" s="26"/>
-      <c r="AF19" s="26" t="s">
+      <c r="AE19" s="35"/>
+      <c r="AF19" s="35" t="s">
         <v>26</v>
       </c>
       <c r="AG19" s="1">
         <v>3</v>
       </c>
-      <c r="AH19" s="26">
+      <c r="AH19" s="35">
         <v>11</v>
       </c>
-      <c r="AI19" s="29"/>
-      <c r="AJ19" s="29">
+      <c r="AI19" s="33"/>
+      <c r="AJ19" s="33">
         <v>207</v>
       </c>
       <c r="AK19" s="1">
@@ -2379,32 +2263,31 @@
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
-      <c r="H20" s="32"/>
-      <c r="I20" s="37" t="s">
-        <v>5</v>
-      </c>
-      <c r="J20" s="37"/>
-      <c r="K20" s="37"/>
-      <c r="L20" s="37" t="s">
+      <c r="I20" s="39" t="s">
+        <v>5</v>
+      </c>
+      <c r="J20" s="39"/>
+      <c r="K20" s="39"/>
+      <c r="L20" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="M20" s="37"/>
-      <c r="N20" s="37"/>
-      <c r="O20" s="35" t="s">
+      <c r="M20" s="39"/>
+      <c r="N20" s="39"/>
+      <c r="O20" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="P20" s="35"/>
-      <c r="Q20" s="35"/>
-      <c r="R20" s="33"/>
-      <c r="V20" s="27"/>
-      <c r="W20" s="28"/>
+      <c r="P20" s="34"/>
+      <c r="Q20" s="34"/>
+      <c r="R20" s="1"/>
+      <c r="V20" s="36"/>
+      <c r="W20" s="37"/>
       <c r="X20" s="14">
         <v>2</v>
       </c>
       <c r="Y20" s="1">
         <v>22</v>
       </c>
-      <c r="Z20" s="29"/>
+      <c r="Z20" s="33"/>
       <c r="AA20" s="1">
         <v>0</v>
       </c>
@@ -2414,14 +2297,14 @@
       <c r="AC20" s="1">
         <v>2.5</v>
       </c>
-      <c r="AE20" s="26"/>
-      <c r="AF20" s="26"/>
+      <c r="AE20" s="35"/>
+      <c r="AF20" s="35"/>
       <c r="AG20" s="1">
         <v>3</v>
       </c>
-      <c r="AH20" s="26"/>
-      <c r="AI20" s="29"/>
-      <c r="AJ20" s="29"/>
+      <c r="AH20" s="35"/>
+      <c r="AI20" s="33"/>
+      <c r="AJ20" s="33"/>
       <c r="AK20" s="1">
         <v>9</v>
       </c>
@@ -2454,43 +2337,43 @@
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
-      <c r="I21" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="J21" s="36" t="s">
-        <v>1</v>
-      </c>
-      <c r="K21" s="38" t="s">
-        <v>2</v>
-      </c>
-      <c r="L21" s="39" t="s">
+      <c r="I21" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="K21" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="L21" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="M21" s="40" t="s">
+      <c r="M21" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="N21" s="38" t="s">
+      <c r="N21" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="O21" s="39" t="s">
+      <c r="O21" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="P21" s="40" t="s">
+      <c r="P21" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="Q21" s="38" t="s">
+      <c r="Q21" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="R21" s="33"/>
-      <c r="V21" s="27"/>
-      <c r="W21" s="28"/>
+      <c r="R21" s="1"/>
+      <c r="V21" s="36"/>
+      <c r="W21" s="37"/>
       <c r="X21" s="1">
         <v>2</v>
       </c>
       <c r="Y21" s="1">
         <v>31</v>
       </c>
-      <c r="Z21" s="29"/>
+      <c r="Z21" s="33"/>
       <c r="AA21" s="1">
         <v>0</v>
       </c>
@@ -2500,14 +2383,14 @@
       <c r="AC21" s="1">
         <v>1.75</v>
       </c>
-      <c r="AE21" s="26"/>
-      <c r="AF21" s="26"/>
+      <c r="AE21" s="35"/>
+      <c r="AF21" s="35"/>
       <c r="AG21" s="1">
         <v>3</v>
       </c>
-      <c r="AH21" s="26"/>
-      <c r="AI21" s="29"/>
-      <c r="AJ21" s="29"/>
+      <c r="AH21" s="35"/>
+      <c r="AI21" s="33"/>
+      <c r="AJ21" s="33"/>
       <c r="AK21" s="1">
         <v>9</v>
       </c>
@@ -2540,46 +2423,46 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
-      <c r="H22" s="48" t="s">
+      <c r="H22" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="I22" s="33">
-        <v>1</v>
-      </c>
-      <c r="J22" s="33">
-        <v>1</v>
-      </c>
-      <c r="K22" s="41">
+      <c r="I22" s="1">
+        <v>1</v>
+      </c>
+      <c r="J22" s="1">
+        <v>1</v>
+      </c>
+      <c r="K22" s="27">
         <v>2.5</v>
       </c>
-      <c r="L22" s="42">
-        <v>0</v>
-      </c>
-      <c r="M22" s="43">
-        <v>0</v>
-      </c>
-      <c r="N22" s="41">
+      <c r="L22" s="6">
+        <v>0</v>
+      </c>
+      <c r="M22" s="7">
+        <v>0</v>
+      </c>
+      <c r="N22" s="27">
         <v>2.5</v>
       </c>
-      <c r="O22" s="39">
-        <v>1</v>
-      </c>
-      <c r="P22" s="40">
-        <v>1</v>
-      </c>
-      <c r="Q22" s="38">
+      <c r="O22" s="25">
+        <v>1</v>
+      </c>
+      <c r="P22" s="26">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="24">
         <f>$K$13-(K22/2)</f>
         <v>3.75</v>
       </c>
-      <c r="V22" s="27"/>
-      <c r="W22" s="28"/>
+      <c r="V22" s="36"/>
+      <c r="W22" s="37"/>
       <c r="X22" s="14">
         <v>2</v>
       </c>
       <c r="Y22" s="1">
         <v>36</v>
       </c>
-      <c r="Z22" s="29"/>
+      <c r="Z22" s="33"/>
       <c r="AA22" s="1">
         <v>0</v>
       </c>
@@ -2589,18 +2472,18 @@
       <c r="AC22" s="1">
         <v>0.75</v>
       </c>
-      <c r="AE22" s="26"/>
-      <c r="AF22" s="26" t="s">
+      <c r="AE22" s="35"/>
+      <c r="AF22" s="35" t="s">
         <v>27</v>
       </c>
       <c r="AG22" s="1">
         <v>3</v>
       </c>
-      <c r="AH22" s="26">
+      <c r="AH22" s="35">
         <v>14</v>
       </c>
-      <c r="AI22" s="29"/>
-      <c r="AJ22" s="29">
+      <c r="AI22" s="33"/>
+      <c r="AJ22" s="33">
         <v>208</v>
       </c>
       <c r="AK22" s="1">
@@ -2635,42 +2518,42 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
-      <c r="H23" s="48" t="s">
+      <c r="H23" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="I23" s="33">
-        <v>9</v>
-      </c>
-      <c r="J23" s="33">
-        <v>9</v>
-      </c>
-      <c r="K23" s="41">
+      <c r="I23" s="1">
+        <v>9</v>
+      </c>
+      <c r="J23" s="1">
+        <v>9</v>
+      </c>
+      <c r="K23" s="27">
         <v>2.5</v>
       </c>
-      <c r="L23" s="42">
-        <v>0</v>
-      </c>
-      <c r="M23" s="43">
-        <v>0</v>
-      </c>
-      <c r="N23" s="41">
+      <c r="L23" s="6">
+        <v>0</v>
+      </c>
+      <c r="M23" s="7">
+        <v>0</v>
+      </c>
+      <c r="N23" s="27">
         <f>K23-K24</f>
         <v>2.5</v>
       </c>
-      <c r="O23" s="39">
-        <v>9</v>
-      </c>
-      <c r="P23" s="40">
-        <v>9</v>
-      </c>
-      <c r="Q23" s="38">
+      <c r="O23" s="25">
+        <v>9</v>
+      </c>
+      <c r="P23" s="26">
+        <v>9</v>
+      </c>
+      <c r="Q23" s="24">
         <f>$K$13-(K23/2)</f>
         <v>3.75</v>
       </c>
-      <c r="V23" s="27" t="s">
+      <c r="V23" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="W23" s="28" t="s">
+      <c r="W23" s="37" t="s">
         <v>63</v>
       </c>
       <c r="X23" s="1">
@@ -2679,7 +2562,7 @@
       <c r="Y23" s="1">
         <v>6</v>
       </c>
-      <c r="Z23" s="29">
+      <c r="Z23" s="33">
         <v>302</v>
       </c>
       <c r="AA23" s="20">
@@ -2691,14 +2574,14 @@
       <c r="AC23" s="1">
         <v>4.25</v>
       </c>
-      <c r="AE23" s="26"/>
-      <c r="AF23" s="26"/>
+      <c r="AE23" s="35"/>
+      <c r="AF23" s="35"/>
       <c r="AG23" s="1">
         <v>3</v>
       </c>
-      <c r="AH23" s="26"/>
-      <c r="AI23" s="29"/>
-      <c r="AJ23" s="29"/>
+      <c r="AH23" s="35"/>
+      <c r="AI23" s="33"/>
+      <c r="AJ23" s="33"/>
       <c r="AK23" s="1">
         <v>9</v>
       </c>
@@ -2736,25 +2619,23 @@
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="33"/>
-      <c r="K24" s="33"/>
-      <c r="L24" s="33"/>
-      <c r="M24" s="33"/>
-      <c r="N24" s="33"/>
-      <c r="O24" s="33"/>
-      <c r="P24" s="33"/>
-      <c r="Q24" s="32"/>
-      <c r="V24" s="27"/>
-      <c r="W24" s="28"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="V24" s="36"/>
+      <c r="W24" s="37"/>
       <c r="X24" s="14">
         <v>2</v>
       </c>
       <c r="Y24" s="1">
         <v>17</v>
       </c>
-      <c r="Z24" s="29"/>
+      <c r="Z24" s="33"/>
       <c r="AA24" s="20">
         <v>10</v>
       </c>
@@ -2764,14 +2645,14 @@
       <c r="AC24" s="1">
         <v>3.25</v>
       </c>
-      <c r="AE24" s="26"/>
-      <c r="AF24" s="26"/>
+      <c r="AE24" s="35"/>
+      <c r="AF24" s="35"/>
       <c r="AG24" s="1">
         <v>3</v>
       </c>
-      <c r="AH24" s="26"/>
-      <c r="AI24" s="29"/>
-      <c r="AJ24" s="29"/>
+      <c r="AH24" s="35"/>
+      <c r="AI24" s="33"/>
+      <c r="AJ24" s="33"/>
       <c r="AK24" s="1">
         <v>9</v>
       </c>
@@ -2806,15 +2687,15 @@
       <c r="F25" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="V25" s="27"/>
-      <c r="W25" s="28"/>
+      <c r="V25" s="36"/>
+      <c r="W25" s="37"/>
       <c r="X25" s="14">
         <v>2</v>
       </c>
       <c r="Y25" s="1">
         <v>26</v>
       </c>
-      <c r="Z25" s="29"/>
+      <c r="Z25" s="33"/>
       <c r="AA25" s="20">
         <v>10</v>
       </c>
@@ -2835,15 +2716,15 @@
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
-      <c r="V26" s="27"/>
-      <c r="W26" s="28"/>
+      <c r="V26" s="36"/>
+      <c r="W26" s="37"/>
       <c r="X26" s="1">
         <v>2</v>
       </c>
       <c r="Y26" s="1">
         <v>32</v>
       </c>
-      <c r="Z26" s="29"/>
+      <c r="Z26" s="33"/>
       <c r="AA26" s="20">
         <v>10</v>
       </c>
@@ -2865,15 +2746,15 @@
       <c r="G27" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="V27" s="27"/>
-      <c r="W27" s="28"/>
+      <c r="V27" s="36"/>
+      <c r="W27" s="37"/>
       <c r="X27" s="14">
         <v>2</v>
       </c>
       <c r="Y27" s="1">
         <v>37</v>
       </c>
-      <c r="Z27" s="29"/>
+      <c r="Z27" s="33"/>
       <c r="AA27" s="20">
         <v>10</v>
       </c>
@@ -2894,10 +2775,10 @@
       <c r="F28" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="V28" s="27" t="s">
+      <c r="V28" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="W28" s="28" t="s">
+      <c r="W28" s="37" t="s">
         <v>65</v>
       </c>
       <c r="X28" s="14">
@@ -2906,7 +2787,7 @@
       <c r="Y28" s="1">
         <v>2</v>
       </c>
-      <c r="Z28" s="29">
+      <c r="Z28" s="33">
         <v>303</v>
       </c>
       <c r="AA28" s="1">
@@ -2920,15 +2801,15 @@
       </c>
     </row>
     <row r="29" spans="2:46" x14ac:dyDescent="0.25">
-      <c r="V29" s="27"/>
-      <c r="W29" s="28"/>
+      <c r="V29" s="36"/>
+      <c r="W29" s="37"/>
       <c r="X29" s="1">
         <v>2</v>
       </c>
       <c r="Y29" s="1">
         <v>14</v>
       </c>
-      <c r="Z29" s="29"/>
+      <c r="Z29" s="33"/>
       <c r="AA29" s="1">
         <v>5</v>
       </c>
@@ -2938,20 +2819,17 @@
       <c r="AC29" s="1">
         <v>3.25</v>
       </c>
-      <c r="AG29" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="30" spans="2:46" x14ac:dyDescent="0.25">
-      <c r="V30" s="27"/>
-      <c r="W30" s="28"/>
+      <c r="V30" s="36"/>
+      <c r="W30" s="37"/>
       <c r="X30" s="14">
         <v>2</v>
       </c>
       <c r="Y30" s="1">
         <v>23</v>
       </c>
-      <c r="Z30" s="29"/>
+      <c r="Z30" s="33"/>
       <c r="AA30" s="1">
         <v>5</v>
       </c>
@@ -2961,20 +2839,17 @@
       <c r="AC30" s="1">
         <v>2.5</v>
       </c>
-      <c r="AG30" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="31" spans="2:46" x14ac:dyDescent="0.25">
-      <c r="V31" s="27"/>
-      <c r="W31" s="28"/>
+      <c r="V31" s="36"/>
+      <c r="W31" s="37"/>
       <c r="X31" s="14">
         <v>2</v>
       </c>
       <c r="Y31" s="1">
         <v>33</v>
       </c>
-      <c r="Z31" s="29"/>
+      <c r="Z31" s="33"/>
       <c r="AA31" s="1">
         <v>5</v>
       </c>
@@ -2984,23 +2859,17 @@
       <c r="AC31" s="1">
         <v>1.75</v>
       </c>
-      <c r="AG31" t="s">
-        <v>76</v>
-      </c>
-      <c r="AK31" t="s">
-        <v>87</v>
-      </c>
     </row>
     <row r="32" spans="2:46" x14ac:dyDescent="0.25">
-      <c r="V32" s="27"/>
-      <c r="W32" s="28"/>
+      <c r="V32" s="36"/>
+      <c r="W32" s="37"/>
       <c r="X32" s="1">
         <v>2</v>
       </c>
       <c r="Y32" s="1">
         <v>38</v>
       </c>
-      <c r="Z32" s="29"/>
+      <c r="Z32" s="33"/>
       <c r="AA32" s="1">
         <v>5</v>
       </c>
@@ -3010,18 +2879,12 @@
       <c r="AC32" s="1">
         <v>0.75</v>
       </c>
-      <c r="AG32" t="s">
-        <v>77</v>
-      </c>
-      <c r="AK32" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="33" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V33" s="27" t="s">
+    </row>
+    <row r="33" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V33" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="W33" s="28" t="s">
+      <c r="W33" s="37" t="s">
         <v>69</v>
       </c>
       <c r="X33" s="14">
@@ -3030,7 +2893,7 @@
       <c r="Y33" s="1">
         <v>4</v>
       </c>
-      <c r="Z33" s="29">
+      <c r="Z33" s="33">
         <v>304</v>
       </c>
       <c r="AA33" s="1">
@@ -3042,23 +2905,17 @@
       <c r="AC33" s="1">
         <v>4.25</v>
       </c>
-      <c r="AG33" t="s">
-        <v>78</v>
-      </c>
-      <c r="AK33" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="34" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V34" s="27"/>
-      <c r="W34" s="28"/>
+    </row>
+    <row r="34" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V34" s="36"/>
+      <c r="W34" s="37"/>
       <c r="X34" s="1">
         <v>2</v>
       </c>
       <c r="Y34" s="1">
         <v>15</v>
       </c>
-      <c r="Z34" s="29"/>
+      <c r="Z34" s="33"/>
       <c r="AA34" s="1">
         <v>5</v>
       </c>
@@ -3068,23 +2925,17 @@
       <c r="AC34" s="1">
         <v>3.25</v>
       </c>
-      <c r="AG34" t="s">
-        <v>79</v>
-      </c>
-      <c r="AK34" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="35" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V35" s="27"/>
-      <c r="W35" s="28"/>
+    </row>
+    <row r="35" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V35" s="36"/>
+      <c r="W35" s="37"/>
       <c r="X35" s="14">
         <v>2</v>
       </c>
       <c r="Y35" s="1">
         <v>24</v>
       </c>
-      <c r="Z35" s="29"/>
+      <c r="Z35" s="33"/>
       <c r="AA35" s="1">
         <v>5</v>
       </c>
@@ -3094,31 +2945,18 @@
       <c r="AC35" s="1">
         <v>2.5</v>
       </c>
-      <c r="AF35" s="24"/>
-      <c r="AG35" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="AH35" s="24"/>
-      <c r="AI35" s="24"/>
-      <c r="AK35" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="36" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="N36" s="32"/>
-      <c r="O36" s="32"/>
-      <c r="P36" s="32"/>
-      <c r="Q36" s="32"/>
-      <c r="R36" s="36"/>
-      <c r="V36" s="27"/>
-      <c r="W36" s="28"/>
+    </row>
+    <row r="36" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="R36" s="9"/>
+      <c r="V36" s="36"/>
+      <c r="W36" s="37"/>
       <c r="X36" s="14">
         <v>2</v>
       </c>
       <c r="Y36" s="1">
         <v>34</v>
       </c>
-      <c r="Z36" s="29"/>
+      <c r="Z36" s="33"/>
       <c r="AA36" s="1">
         <v>5</v>
       </c>
@@ -3128,23 +2966,17 @@
       <c r="AC36" s="1">
         <v>1.75</v>
       </c>
-      <c r="AG36" t="s">
-        <v>81</v>
-      </c>
-      <c r="AK36" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="37" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V37" s="27"/>
-      <c r="W37" s="28"/>
+    </row>
+    <row r="37" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V37" s="36"/>
+      <c r="W37" s="37"/>
       <c r="X37" s="1">
         <v>2</v>
       </c>
       <c r="Y37" s="1">
         <v>39</v>
       </c>
-      <c r="Z37" s="29"/>
+      <c r="Z37" s="33"/>
       <c r="AA37" s="1">
         <v>5</v>
       </c>
@@ -3154,188 +2986,161 @@
       <c r="AC37" s="1">
         <v>0.75</v>
       </c>
-      <c r="AG37" t="s">
-        <v>82</v>
-      </c>
-      <c r="AK37" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="38" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V38" s="27" t="s">
+    </row>
+    <row r="38" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V38" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="W38" s="28" t="s">
+      <c r="W38" s="37" t="s">
         <v>70</v>
       </c>
       <c r="X38" s="14">
         <v>2</v>
       </c>
-      <c r="Y38" s="26">
+      <c r="Y38" s="35">
         <v>3</v>
       </c>
-      <c r="Z38" s="29">
+      <c r="Z38" s="33">
         <v>305</v>
       </c>
-      <c r="AA38" s="26">
-        <v>5</v>
-      </c>
-      <c r="AB38" s="26">
-        <v>5</v>
-      </c>
-      <c r="AC38" s="26">
-        <v>5</v>
-      </c>
-      <c r="AG38" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="39" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V39" s="27"/>
-      <c r="W39" s="28"/>
+      <c r="AA38" s="35">
+        <v>5</v>
+      </c>
+      <c r="AB38" s="35">
+        <v>5</v>
+      </c>
+      <c r="AC38" s="35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V39" s="36"/>
+      <c r="W39" s="37"/>
       <c r="X39" s="1">
         <v>2</v>
       </c>
-      <c r="Y39" s="26"/>
-      <c r="Z39" s="29"/>
-      <c r="AA39" s="26"/>
-      <c r="AB39" s="26"/>
-      <c r="AC39" s="26"/>
-      <c r="AF39" s="24"/>
-      <c r="AG39" s="24" t="s">
-        <v>84</v>
-      </c>
-      <c r="AH39" s="24"/>
-      <c r="AI39" s="24"/>
-    </row>
-    <row r="40" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V40" s="27"/>
-      <c r="W40" s="28"/>
+      <c r="Y39" s="35"/>
+      <c r="Z39" s="33"/>
+      <c r="AA39" s="35"/>
+      <c r="AB39" s="35"/>
+      <c r="AC39" s="35"/>
+    </row>
+    <row r="40" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V40" s="36"/>
+      <c r="W40" s="37"/>
       <c r="X40" s="14">
         <v>2</v>
       </c>
-      <c r="Y40" s="26"/>
-      <c r="Z40" s="29"/>
-      <c r="AA40" s="26"/>
-      <c r="AB40" s="26"/>
-      <c r="AC40" s="26"/>
-      <c r="AG40" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="41" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V41" s="27"/>
-      <c r="W41" s="28"/>
+      <c r="Y40" s="35"/>
+      <c r="Z40" s="33"/>
+      <c r="AA40" s="35"/>
+      <c r="AB40" s="35"/>
+      <c r="AC40" s="35"/>
+    </row>
+    <row r="41" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V41" s="36"/>
+      <c r="W41" s="37"/>
       <c r="X41" s="14">
         <v>2</v>
       </c>
-      <c r="Y41" s="26"/>
-      <c r="Z41" s="29"/>
-      <c r="AA41" s="26"/>
-      <c r="AB41" s="26"/>
-      <c r="AC41" s="26"/>
-      <c r="AG41" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="42" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V42" s="27"/>
-      <c r="W42" s="28"/>
+      <c r="Y41" s="35"/>
+      <c r="Z41" s="33"/>
+      <c r="AA41" s="35"/>
+      <c r="AB41" s="35"/>
+      <c r="AC41" s="35"/>
+    </row>
+    <row r="42" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V42" s="36"/>
+      <c r="W42" s="37"/>
       <c r="X42" s="1">
         <v>2</v>
       </c>
-      <c r="Y42" s="26"/>
-      <c r="Z42" s="29"/>
-      <c r="AA42" s="26"/>
-      <c r="AB42" s="26"/>
-      <c r="AC42" s="26"/>
-    </row>
-    <row r="43" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V43" s="27" t="s">
+      <c r="Y42" s="35"/>
+      <c r="Z42" s="33"/>
+      <c r="AA42" s="35"/>
+      <c r="AB42" s="35"/>
+      <c r="AC42" s="35"/>
+    </row>
+    <row r="43" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V43" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="W43" s="28" t="s">
+      <c r="W43" s="37" t="s">
         <v>73</v>
       </c>
       <c r="X43" s="14">
         <v>2</v>
       </c>
-      <c r="Y43" s="26">
+      <c r="Y43" s="35">
         <v>40</v>
       </c>
-      <c r="Z43" s="29">
+      <c r="Z43" s="33">
         <v>306</v>
       </c>
-      <c r="AA43" s="26">
-        <v>5</v>
-      </c>
-      <c r="AB43" s="26">
-        <v>5</v>
-      </c>
-      <c r="AC43" s="26">
+      <c r="AA43" s="35">
+        <v>5</v>
+      </c>
+      <c r="AB43" s="35">
+        <v>5</v>
+      </c>
+      <c r="AC43" s="35">
         <v>0</v>
       </c>
       <c r="AE43" s="1"/>
-      <c r="AH43" s="1"/>
-      <c r="AI43" s="1"/>
-      <c r="AJ43" s="1"/>
-      <c r="AK43" s="1"/>
-      <c r="AL43" s="1"/>
-      <c r="AM43" s="1"/>
-    </row>
-    <row r="44" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V44" s="27"/>
-      <c r="W44" s="28"/>
+    </row>
+    <row r="44" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V44" s="36"/>
+      <c r="W44" s="37"/>
       <c r="X44" s="1">
         <v>2</v>
       </c>
-      <c r="Y44" s="26"/>
-      <c r="Z44" s="29"/>
-      <c r="AA44" s="26"/>
-      <c r="AB44" s="26"/>
-      <c r="AC44" s="26"/>
+      <c r="Y44" s="35"/>
+      <c r="Z44" s="33"/>
+      <c r="AA44" s="35"/>
+      <c r="AB44" s="35"/>
+      <c r="AC44" s="35"/>
       <c r="AE44" s="1"/>
     </row>
-    <row r="45" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V45" s="27"/>
-      <c r="W45" s="28"/>
+    <row r="45" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V45" s="36"/>
+      <c r="W45" s="37"/>
       <c r="X45" s="14">
         <v>2</v>
       </c>
-      <c r="Y45" s="26"/>
-      <c r="Z45" s="29"/>
-      <c r="AA45" s="26"/>
-      <c r="AB45" s="26"/>
-      <c r="AC45" s="26"/>
+      <c r="Y45" s="35"/>
+      <c r="Z45" s="33"/>
+      <c r="AA45" s="35"/>
+      <c r="AB45" s="35"/>
+      <c r="AC45" s="35"/>
       <c r="AE45" s="1"/>
     </row>
-    <row r="46" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V46" s="27"/>
-      <c r="W46" s="28"/>
+    <row r="46" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V46" s="36"/>
+      <c r="W46" s="37"/>
       <c r="X46" s="14">
         <v>2</v>
       </c>
-      <c r="Y46" s="26"/>
-      <c r="Z46" s="29"/>
-      <c r="AA46" s="26"/>
-      <c r="AB46" s="26"/>
-      <c r="AC46" s="26"/>
+      <c r="Y46" s="35"/>
+      <c r="Z46" s="33"/>
+      <c r="AA46" s="35"/>
+      <c r="AB46" s="35"/>
+      <c r="AC46" s="35"/>
       <c r="AE46" s="1"/>
     </row>
-    <row r="47" spans="14:39" x14ac:dyDescent="0.25">
-      <c r="V47" s="27"/>
-      <c r="W47" s="28"/>
+    <row r="47" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="V47" s="36"/>
+      <c r="W47" s="37"/>
       <c r="X47" s="1">
         <v>2</v>
       </c>
-      <c r="Y47" s="26"/>
-      <c r="Z47" s="29"/>
-      <c r="AA47" s="26"/>
-      <c r="AB47" s="26"/>
-      <c r="AC47" s="26"/>
+      <c r="Y47" s="35"/>
+      <c r="Z47" s="33"/>
+      <c r="AA47" s="35"/>
+      <c r="AB47" s="35"/>
+      <c r="AC47" s="35"/>
       <c r="AE47" s="1"/>
     </row>
-    <row r="48" spans="14:39" x14ac:dyDescent="0.25">
+    <row r="48" spans="18:31" x14ac:dyDescent="0.25">
       <c r="V48" s="22"/>
       <c r="W48" s="20"/>
       <c r="X48" s="1"/>
@@ -3420,39 +3225,13 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="AJ22:AJ24"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="AJ7:AJ9"/>
-    <mergeCell ref="AJ10:AJ12"/>
-    <mergeCell ref="AJ13:AJ15"/>
-    <mergeCell ref="AJ16:AJ18"/>
-    <mergeCell ref="AJ19:AJ21"/>
-    <mergeCell ref="AI7:AI15"/>
-    <mergeCell ref="AI16:AI24"/>
-    <mergeCell ref="AC38:AC42"/>
-    <mergeCell ref="AA43:AA47"/>
-    <mergeCell ref="AB43:AB47"/>
-    <mergeCell ref="AC43:AC47"/>
-    <mergeCell ref="Y43:Y47"/>
-    <mergeCell ref="V43:V47"/>
-    <mergeCell ref="W43:W47"/>
-    <mergeCell ref="Z43:Z47"/>
-    <mergeCell ref="AA38:AA42"/>
-    <mergeCell ref="AB38:AB42"/>
-    <mergeCell ref="V33:V37"/>
-    <mergeCell ref="W33:W37"/>
-    <mergeCell ref="Z33:Z37"/>
-    <mergeCell ref="V38:V42"/>
-    <mergeCell ref="W38:W42"/>
-    <mergeCell ref="Y38:Y42"/>
-    <mergeCell ref="Z38:Z42"/>
-    <mergeCell ref="AH22:AH24"/>
-    <mergeCell ref="Z18:Z22"/>
-    <mergeCell ref="W18:W22"/>
-    <mergeCell ref="V18:V22"/>
-    <mergeCell ref="V23:V27"/>
-    <mergeCell ref="W23:W27"/>
-    <mergeCell ref="Z23:Z27"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="O11:Q11"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="L20:N20"/>
+    <mergeCell ref="O20:Q20"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="I11:K11"/>
     <mergeCell ref="AH7:AH9"/>
     <mergeCell ref="AF7:AF9"/>
     <mergeCell ref="V28:V32"/>
@@ -3469,13 +3248,39 @@
     <mergeCell ref="AF19:AF21"/>
     <mergeCell ref="AH19:AH21"/>
     <mergeCell ref="AF22:AF24"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="O11:Q11"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="L20:N20"/>
-    <mergeCell ref="O20:Q20"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="AH22:AH24"/>
+    <mergeCell ref="Z18:Z22"/>
+    <mergeCell ref="W18:W22"/>
+    <mergeCell ref="V18:V22"/>
+    <mergeCell ref="V23:V27"/>
+    <mergeCell ref="W23:W27"/>
+    <mergeCell ref="Z23:Z27"/>
+    <mergeCell ref="V33:V37"/>
+    <mergeCell ref="W33:W37"/>
+    <mergeCell ref="Z33:Z37"/>
+    <mergeCell ref="V38:V42"/>
+    <mergeCell ref="W38:W42"/>
+    <mergeCell ref="Y38:Y42"/>
+    <mergeCell ref="Z38:Z42"/>
+    <mergeCell ref="V43:V47"/>
+    <mergeCell ref="W43:W47"/>
+    <mergeCell ref="Z43:Z47"/>
+    <mergeCell ref="AA38:AA42"/>
+    <mergeCell ref="AB38:AB42"/>
+    <mergeCell ref="AC38:AC42"/>
+    <mergeCell ref="AA43:AA47"/>
+    <mergeCell ref="AB43:AB47"/>
+    <mergeCell ref="AC43:AC47"/>
+    <mergeCell ref="Y43:Y47"/>
+    <mergeCell ref="AJ22:AJ24"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="AJ7:AJ9"/>
+    <mergeCell ref="AJ10:AJ12"/>
+    <mergeCell ref="AJ13:AJ15"/>
+    <mergeCell ref="AJ16:AJ18"/>
+    <mergeCell ref="AJ19:AJ21"/>
+    <mergeCell ref="AI7:AI15"/>
+    <mergeCell ref="AI16:AI24"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>